<commit_message>
fix(import): garantir leitura, persistência na BD e exibição do Vendedor e Notas Motorista na importação Excel e Georreferenciação
</commit_message>
<xml_diff>
--- a/Ficheiros EXCEL/AUC/GeoRoute_Completo_SoRotas_2026-08-25.xlsx
+++ b/Ficheiros EXCEL/AUC/GeoRoute_Completo_SoRotas_2026-08-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo\.gemini\antigravity\playground\core-omega\PRJT_GEO\Ficheiros EXCEL\AUC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8FED28-5992-464E-A5C3-0C4A0A9DE957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A59FA9-4575-4C98-B084-2638A3037944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3134" uniqueCount="1064">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3135" uniqueCount="1064">
   <si>
     <t>Nome_Armazem</t>
   </si>
@@ -3224,8 +3224,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00\ \€"/>
+    <numFmt numFmtId="166" formatCode="h:mm;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -3351,7 +3352,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3406,6 +3407,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7969,10 +7976,10 @@
       <c r="K2" s="6">
         <v>1</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N2" s="5"/>
@@ -8026,10 +8033,10 @@
       <c r="K3" s="9">
         <v>1</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N3" s="8"/>
@@ -8083,10 +8090,10 @@
       <c r="K4" s="6">
         <v>1</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="M4" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N4" s="5"/>
@@ -8140,10 +8147,10 @@
       <c r="K5" s="9">
         <v>1</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="L5" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="M5" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N5" s="8"/>
@@ -8197,10 +8204,10 @@
       <c r="K6" s="6">
         <v>1</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="M6" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N6" s="5"/>
@@ -8254,10 +8261,10 @@
       <c r="K7" s="9">
         <v>1</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="L7" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="M7" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N7" s="8"/>
@@ -8311,10 +8318,10 @@
       <c r="K8" s="6">
         <v>1</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="L8" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M8" s="5" t="s">
+      <c r="M8" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N8" s="5"/>
@@ -8368,10 +8375,10 @@
       <c r="K9" s="9">
         <v>1</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="M9" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N9" s="8"/>
@@ -8425,10 +8432,10 @@
       <c r="K10" s="6">
         <v>1</v>
       </c>
-      <c r="L10" s="5" t="s">
+      <c r="L10" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M10" s="5" t="s">
+      <c r="M10" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N10" s="5"/>
@@ -8482,10 +8489,10 @@
       <c r="K11" s="9">
         <v>1</v>
       </c>
-      <c r="L11" s="8" t="s">
+      <c r="L11" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M11" s="8" t="s">
+      <c r="M11" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N11" s="8"/>
@@ -8539,10 +8546,10 @@
       <c r="K12" s="6">
         <v>1</v>
       </c>
-      <c r="L12" s="5" t="s">
+      <c r="L12" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M12" s="5" t="s">
+      <c r="M12" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N12" s="5"/>
@@ -8596,10 +8603,10 @@
       <c r="K13" s="9">
         <v>1</v>
       </c>
-      <c r="L13" s="8" t="s">
+      <c r="L13" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="M13" s="8" t="s">
+      <c r="M13" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N13" s="8"/>
@@ -8653,10 +8660,10 @@
       <c r="K14" s="6">
         <v>1</v>
       </c>
-      <c r="L14" s="5" t="s">
+      <c r="L14" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="M14" s="5" t="s">
+      <c r="M14" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N14" s="5"/>
@@ -8710,10 +8717,10 @@
       <c r="K15" s="9">
         <v>1</v>
       </c>
-      <c r="L15" s="8" t="s">
+      <c r="L15" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M15" s="8" t="s">
+      <c r="M15" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N15" s="8"/>
@@ -8767,10 +8774,10 @@
       <c r="K16" s="6">
         <v>1</v>
       </c>
-      <c r="L16" s="5" t="s">
+      <c r="L16" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="M16" s="5" t="s">
+      <c r="M16" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N16" s="5"/>
@@ -8824,10 +8831,10 @@
       <c r="K17" s="9">
         <v>1</v>
       </c>
-      <c r="L17" s="8" t="s">
+      <c r="L17" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="M17" s="8" t="s">
+      <c r="M17" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N17" s="8"/>
@@ -8881,10 +8888,10 @@
       <c r="K18" s="6">
         <v>1</v>
       </c>
-      <c r="L18" s="5" t="s">
+      <c r="L18" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="M18" s="5" t="s">
+      <c r="M18" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N18" s="5"/>
@@ -8938,10 +8945,10 @@
       <c r="K19" s="9">
         <v>1</v>
       </c>
-      <c r="L19" s="8" t="s">
+      <c r="L19" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M19" s="8" t="s">
+      <c r="M19" s="20" t="s">
         <v>284</v>
       </c>
       <c r="N19" s="8"/>
@@ -8995,10 +9002,10 @@
       <c r="K20" s="6">
         <v>1</v>
       </c>
-      <c r="L20" s="5" t="s">
+      <c r="L20" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M20" s="5" t="s">
+      <c r="M20" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N20" s="5"/>
@@ -9052,10 +9059,10 @@
       <c r="K21" s="9">
         <v>1</v>
       </c>
-      <c r="L21" s="8" t="s">
+      <c r="L21" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M21" s="8" t="s">
+      <c r="M21" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N21" s="8"/>
@@ -9109,10 +9116,10 @@
       <c r="K22" s="6">
         <v>1</v>
       </c>
-      <c r="L22" s="5" t="s">
+      <c r="L22" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M22" s="5" t="s">
+      <c r="M22" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N22" s="5"/>
@@ -9166,10 +9173,10 @@
       <c r="K23" s="9">
         <v>1</v>
       </c>
-      <c r="L23" s="8" t="s">
+      <c r="L23" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M23" s="8" t="s">
+      <c r="M23" s="20" t="s">
         <v>284</v>
       </c>
       <c r="N23" s="8"/>
@@ -9223,10 +9230,10 @@
       <c r="K24" s="6">
         <v>1</v>
       </c>
-      <c r="L24" s="5" t="s">
+      <c r="L24" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M24" s="5" t="s">
+      <c r="M24" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N24" s="5"/>
@@ -9280,10 +9287,10 @@
       <c r="K25" s="9">
         <v>1</v>
       </c>
-      <c r="L25" s="8" t="s">
+      <c r="L25" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M25" s="8" t="s">
+      <c r="M25" s="20" t="s">
         <v>284</v>
       </c>
       <c r="N25" s="8"/>
@@ -9337,10 +9344,10 @@
       <c r="K26" s="6">
         <v>1</v>
       </c>
-      <c r="L26" s="5" t="s">
+      <c r="L26" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M26" s="5" t="s">
+      <c r="M26" s="19" t="s">
         <v>284</v>
       </c>
       <c r="N26" s="5"/>
@@ -9394,10 +9401,10 @@
       <c r="K27" s="9">
         <v>1</v>
       </c>
-      <c r="L27" s="8" t="s">
+      <c r="L27" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M27" s="8" t="s">
+      <c r="M27" s="20" t="s">
         <v>284</v>
       </c>
       <c r="N27" s="8"/>
@@ -9451,10 +9458,10 @@
       <c r="K28" s="6">
         <v>1</v>
       </c>
-      <c r="L28" s="5" t="s">
+      <c r="L28" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="M28" s="5" t="s">
+      <c r="M28" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N28" s="5"/>
@@ -9508,10 +9515,10 @@
       <c r="K29" s="9">
         <v>1</v>
       </c>
-      <c r="L29" s="8" t="s">
+      <c r="L29" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M29" s="8" t="s">
+      <c r="M29" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N29" s="8"/>
@@ -9565,10 +9572,10 @@
       <c r="K30" s="6">
         <v>1</v>
       </c>
-      <c r="L30" s="5" t="s">
+      <c r="L30" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M30" s="5" t="s">
+      <c r="M30" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N30" s="5"/>
@@ -9622,10 +9629,10 @@
       <c r="K31" s="9">
         <v>1</v>
       </c>
-      <c r="L31" s="8" t="s">
+      <c r="L31" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M31" s="8" t="s">
+      <c r="M31" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N31" s="8"/>
@@ -9679,10 +9686,10 @@
       <c r="K32" s="6">
         <v>1</v>
       </c>
-      <c r="L32" s="5" t="s">
+      <c r="L32" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M32" s="5" t="s">
+      <c r="M32" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N32" s="5"/>
@@ -9736,10 +9743,10 @@
       <c r="K33" s="9">
         <v>1</v>
       </c>
-      <c r="L33" s="8" t="s">
+      <c r="L33" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M33" s="8" t="s">
+      <c r="M33" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N33" s="8"/>
@@ -9793,10 +9800,10 @@
       <c r="K34" s="6">
         <v>1</v>
       </c>
-      <c r="L34" s="5" t="s">
+      <c r="L34" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M34" s="5" t="s">
+      <c r="M34" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N34" s="5"/>
@@ -9850,10 +9857,10 @@
       <c r="K35" s="9">
         <v>1</v>
       </c>
-      <c r="L35" s="8" t="s">
+      <c r="L35" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M35" s="8" t="s">
+      <c r="M35" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N35" s="8"/>
@@ -9907,10 +9914,10 @@
       <c r="K36" s="6">
         <v>1</v>
       </c>
-      <c r="L36" s="5" t="s">
+      <c r="L36" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M36" s="5" t="s">
+      <c r="M36" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N36" s="5"/>
@@ -9964,10 +9971,10 @@
       <c r="K37" s="9">
         <v>1</v>
       </c>
-      <c r="L37" s="8" t="s">
+      <c r="L37" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M37" s="8" t="s">
+      <c r="M37" s="20" t="s">
         <v>284</v>
       </c>
       <c r="N37" s="8"/>
@@ -10021,10 +10028,10 @@
       <c r="K38" s="6">
         <v>1</v>
       </c>
-      <c r="L38" s="5" t="s">
+      <c r="L38" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M38" s="5" t="s">
+      <c r="M38" s="19" t="s">
         <v>284</v>
       </c>
       <c r="N38" s="5"/>
@@ -10078,10 +10085,10 @@
       <c r="K39" s="9">
         <v>1</v>
       </c>
-      <c r="L39" s="8" t="s">
+      <c r="L39" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M39" s="8" t="s">
+      <c r="M39" s="20" t="s">
         <v>284</v>
       </c>
       <c r="N39" s="8"/>
@@ -10135,10 +10142,10 @@
       <c r="K40" s="6">
         <v>1</v>
       </c>
-      <c r="L40" s="5" t="s">
+      <c r="L40" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M40" s="5" t="s">
+      <c r="M40" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N40" s="5"/>
@@ -10192,10 +10199,10 @@
       <c r="K41" s="9">
         <v>1</v>
       </c>
-      <c r="L41" s="8" t="s">
+      <c r="L41" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M41" s="8" t="s">
+      <c r="M41" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N41" s="8"/>
@@ -10249,10 +10256,10 @@
       <c r="K42" s="6">
         <v>1</v>
       </c>
-      <c r="L42" s="5" t="s">
+      <c r="L42" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M42" s="5" t="s">
+      <c r="M42" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N42" s="5"/>
@@ -10306,10 +10313,10 @@
       <c r="K43" s="9">
         <v>1</v>
       </c>
-      <c r="L43" s="8" t="s">
+      <c r="L43" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M43" s="8" t="s">
+      <c r="M43" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N43" s="8"/>
@@ -10363,10 +10370,10 @@
       <c r="K44" s="6">
         <v>1</v>
       </c>
-      <c r="L44" s="5" t="s">
+      <c r="L44" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M44" s="5" t="s">
+      <c r="M44" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N44" s="5"/>
@@ -10420,10 +10427,10 @@
       <c r="K45" s="9">
         <v>1</v>
       </c>
-      <c r="L45" s="8" t="s">
+      <c r="L45" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M45" s="8" t="s">
+      <c r="M45" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N45" s="8"/>
@@ -10477,10 +10484,10 @@
       <c r="K46" s="6">
         <v>1</v>
       </c>
-      <c r="L46" s="5" t="s">
+      <c r="L46" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M46" s="5" t="s">
+      <c r="M46" s="19" t="s">
         <v>284</v>
       </c>
       <c r="N46" s="5"/>
@@ -10534,10 +10541,10 @@
       <c r="K47" s="9">
         <v>1</v>
       </c>
-      <c r="L47" s="8" t="s">
+      <c r="L47" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M47" s="8" t="s">
+      <c r="M47" s="20" t="s">
         <v>284</v>
       </c>
       <c r="N47" s="8"/>
@@ -10591,10 +10598,10 @@
       <c r="K48" s="6">
         <v>1</v>
       </c>
-      <c r="L48" s="5" t="s">
+      <c r="L48" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M48" s="5" t="s">
+      <c r="M48" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N48" s="5"/>
@@ -10648,10 +10655,10 @@
       <c r="K49" s="9">
         <v>1</v>
       </c>
-      <c r="L49" s="8" t="s">
+      <c r="L49" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M49" s="8" t="s">
+      <c r="M49" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N49" s="8"/>
@@ -10705,10 +10712,10 @@
       <c r="K50" s="6">
         <v>1</v>
       </c>
-      <c r="L50" s="5" t="s">
+      <c r="L50" s="19" t="s">
         <v>426</v>
       </c>
-      <c r="M50" s="5" t="s">
+      <c r="M50" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N50" s="5"/>
@@ -10762,10 +10769,10 @@
       <c r="K51" s="9">
         <v>1</v>
       </c>
-      <c r="L51" s="8" t="s">
+      <c r="L51" s="20" t="s">
         <v>426</v>
       </c>
-      <c r="M51" s="8" t="s">
+      <c r="M51" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N51" s="8"/>
@@ -10819,10 +10826,10 @@
       <c r="K52" s="6">
         <v>1</v>
       </c>
-      <c r="L52" s="5" t="s">
+      <c r="L52" s="19" t="s">
         <v>437</v>
       </c>
-      <c r="M52" s="5" t="s">
+      <c r="M52" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N52" s="5"/>
@@ -10876,10 +10883,10 @@
       <c r="K53" s="9">
         <v>1</v>
       </c>
-      <c r="L53" s="8" t="s">
+      <c r="L53" s="20" t="s">
         <v>437</v>
       </c>
-      <c r="M53" s="8" t="s">
+      <c r="M53" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N53" s="8"/>
@@ -10933,10 +10940,10 @@
       <c r="K54" s="6">
         <v>1</v>
       </c>
-      <c r="L54" s="5" t="s">
+      <c r="L54" s="19" t="s">
         <v>437</v>
       </c>
-      <c r="M54" s="5" t="s">
+      <c r="M54" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N54" s="5"/>
@@ -10990,10 +10997,10 @@
       <c r="K55" s="9">
         <v>1</v>
       </c>
-      <c r="L55" s="8" t="s">
+      <c r="L55" s="20" t="s">
         <v>437</v>
       </c>
-      <c r="M55" s="8" t="s">
+      <c r="M55" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N55" s="8"/>
@@ -11047,10 +11054,10 @@
       <c r="K56" s="6">
         <v>1</v>
       </c>
-      <c r="L56" s="5" t="s">
+      <c r="L56" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="M56" s="5" t="s">
+      <c r="M56" s="19" t="s">
         <v>458</v>
       </c>
       <c r="N56" s="5"/>
@@ -11104,10 +11111,10 @@
       <c r="K57" s="9">
         <v>1</v>
       </c>
-      <c r="L57" s="8" t="s">
+      <c r="L57" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="M57" s="8" t="s">
+      <c r="M57" s="20" t="s">
         <v>458</v>
       </c>
       <c r="N57" s="8"/>
@@ -11161,10 +11168,10 @@
       <c r="K58" s="6">
         <v>1</v>
       </c>
-      <c r="L58" s="5" t="s">
+      <c r="L58" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="M58" s="5" t="s">
+      <c r="M58" s="19" t="s">
         <v>458</v>
       </c>
       <c r="N58" s="5"/>
@@ -11218,10 +11225,10 @@
       <c r="K59" s="9">
         <v>1</v>
       </c>
-      <c r="L59" s="8" t="s">
+      <c r="L59" s="20" t="s">
         <v>473</v>
       </c>
-      <c r="M59" s="8" t="s">
+      <c r="M59" s="20" t="s">
         <v>474</v>
       </c>
       <c r="N59" s="8"/>
@@ -11275,10 +11282,10 @@
       <c r="K60" s="6">
         <v>1</v>
       </c>
-      <c r="L60" s="5" t="s">
+      <c r="L60" s="19" t="s">
         <v>473</v>
       </c>
-      <c r="M60" s="5" t="s">
+      <c r="M60" s="19" t="s">
         <v>474</v>
       </c>
       <c r="N60" s="5"/>
@@ -11332,10 +11339,10 @@
       <c r="K61" s="9">
         <v>1</v>
       </c>
-      <c r="L61" s="8" t="s">
+      <c r="L61" s="20" t="s">
         <v>473</v>
       </c>
-      <c r="M61" s="8" t="s">
+      <c r="M61" s="20" t="s">
         <v>474</v>
       </c>
       <c r="N61" s="8"/>
@@ -11389,10 +11396,10 @@
       <c r="K62" s="6">
         <v>1</v>
       </c>
-      <c r="L62" s="5" t="s">
+      <c r="L62" s="19" t="s">
         <v>473</v>
       </c>
-      <c r="M62" s="5" t="s">
+      <c r="M62" s="19" t="s">
         <v>474</v>
       </c>
       <c r="N62" s="5"/>
@@ -11446,10 +11453,10 @@
       <c r="K63" s="9">
         <v>1</v>
       </c>
-      <c r="L63" s="8" t="s">
+      <c r="L63" s="20" t="s">
         <v>473</v>
       </c>
-      <c r="M63" s="8" t="s">
+      <c r="M63" s="20" t="s">
         <v>474</v>
       </c>
       <c r="N63" s="8"/>
@@ -11503,10 +11510,10 @@
       <c r="K64" s="6">
         <v>1</v>
       </c>
-      <c r="L64" s="5" t="s">
+      <c r="L64" s="19" t="s">
         <v>473</v>
       </c>
-      <c r="M64" s="5" t="s">
+      <c r="M64" s="19" t="s">
         <v>474</v>
       </c>
       <c r="N64" s="5"/>
@@ -11560,10 +11567,10 @@
       <c r="K65" s="9">
         <v>1</v>
       </c>
-      <c r="L65" s="8" t="s">
+      <c r="L65" s="20" t="s">
         <v>473</v>
       </c>
-      <c r="M65" s="8" t="s">
+      <c r="M65" s="20" t="s">
         <v>474</v>
       </c>
       <c r="N65" s="8"/>
@@ -11617,10 +11624,10 @@
       <c r="K66" s="6">
         <v>1</v>
       </c>
-      <c r="L66" s="5" t="s">
+      <c r="L66" s="19" t="s">
         <v>509</v>
       </c>
-      <c r="M66" s="5" t="s">
+      <c r="M66" s="19" t="s">
         <v>510</v>
       </c>
       <c r="N66" s="5"/>
@@ -11674,10 +11681,10 @@
       <c r="K67" s="9">
         <v>1</v>
       </c>
-      <c r="L67" s="8" t="s">
+      <c r="L67" s="20" t="s">
         <v>509</v>
       </c>
-      <c r="M67" s="8" t="s">
+      <c r="M67" s="20" t="s">
         <v>510</v>
       </c>
       <c r="N67" s="8"/>
@@ -11731,10 +11738,10 @@
       <c r="K68" s="6">
         <v>1</v>
       </c>
-      <c r="L68" s="5" t="s">
+      <c r="L68" s="19" t="s">
         <v>509</v>
       </c>
-      <c r="M68" s="5" t="s">
+      <c r="M68" s="19" t="s">
         <v>510</v>
       </c>
       <c r="N68" s="5"/>
@@ -11788,10 +11795,10 @@
       <c r="K69" s="9">
         <v>1</v>
       </c>
-      <c r="L69" s="8" t="s">
+      <c r="L69" s="20" t="s">
         <v>509</v>
       </c>
-      <c r="M69" s="8" t="s">
+      <c r="M69" s="20" t="s">
         <v>510</v>
       </c>
       <c r="N69" s="8"/>
@@ -11845,10 +11852,10 @@
       <c r="K70" s="6">
         <v>1</v>
       </c>
-      <c r="L70" s="5" t="s">
+      <c r="L70" s="19" t="s">
         <v>509</v>
       </c>
-      <c r="M70" s="5" t="s">
+      <c r="M70" s="19" t="s">
         <v>510</v>
       </c>
       <c r="N70" s="5"/>
@@ -11902,10 +11909,10 @@
       <c r="K71" s="9">
         <v>1</v>
       </c>
-      <c r="L71" s="8" t="s">
+      <c r="L71" s="20" t="s">
         <v>509</v>
       </c>
-      <c r="M71" s="8" t="s">
+      <c r="M71" s="20" t="s">
         <v>510</v>
       </c>
       <c r="N71" s="8"/>
@@ -11959,10 +11966,10 @@
       <c r="K72" s="6">
         <v>1</v>
       </c>
-      <c r="L72" s="5" t="s">
+      <c r="L72" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M72" s="5" t="s">
+      <c r="M72" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N72" s="5"/>
@@ -12016,10 +12023,10 @@
       <c r="K73" s="9">
         <v>1</v>
       </c>
-      <c r="L73" s="8" t="s">
+      <c r="L73" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M73" s="8" t="s">
+      <c r="M73" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N73" s="8"/>
@@ -12073,10 +12080,10 @@
       <c r="K74" s="6">
         <v>1</v>
       </c>
-      <c r="L74" s="5" t="s">
+      <c r="L74" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="M74" s="5" t="s">
+      <c r="M74" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N74" s="5"/>
@@ -12130,10 +12137,10 @@
       <c r="K75" s="9">
         <v>1</v>
       </c>
-      <c r="L75" s="8" t="s">
+      <c r="L75" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="M75" s="8" t="s">
+      <c r="M75" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N75" s="8"/>
@@ -12187,10 +12194,10 @@
       <c r="K76" s="6">
         <v>1</v>
       </c>
-      <c r="L76" s="5" t="s">
+      <c r="L76" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="M76" s="5" t="s">
+      <c r="M76" s="19" t="s">
         <v>215</v>
       </c>
       <c r="N76" s="5"/>
@@ -12244,10 +12251,10 @@
       <c r="K77" s="9">
         <v>1</v>
       </c>
-      <c r="L77" s="8" t="s">
+      <c r="L77" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="M77" s="8" t="s">
+      <c r="M77" s="20" t="s">
         <v>215</v>
       </c>
       <c r="N77" s="8"/>
@@ -12301,10 +12308,10 @@
       <c r="K78" s="6">
         <v>1</v>
       </c>
-      <c r="L78" s="5" t="s">
+      <c r="L78" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M78" s="5" t="s">
+      <c r="M78" s="19" t="s">
         <v>458</v>
       </c>
       <c r="N78" s="5"/>
@@ -12358,10 +12365,10 @@
       <c r="K79" s="9">
         <v>1</v>
       </c>
-      <c r="L79" s="8" t="s">
+      <c r="L79" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M79" s="8" t="s">
+      <c r="M79" s="20" t="s">
         <v>458</v>
       </c>
       <c r="N79" s="8"/>
@@ -12415,10 +12422,10 @@
       <c r="K80" s="6">
         <v>1</v>
       </c>
-      <c r="L80" s="5" t="s">
+      <c r="L80" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M80" s="5" t="s">
+      <c r="M80" s="19" t="s">
         <v>458</v>
       </c>
       <c r="N80" s="5"/>
@@ -12472,10 +12479,10 @@
       <c r="K81" s="9">
         <v>1</v>
       </c>
-      <c r="L81" s="8" t="s">
+      <c r="L81" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M81" s="8" t="s">
+      <c r="M81" s="20" t="s">
         <v>458</v>
       </c>
       <c r="N81" s="8"/>
@@ -12529,10 +12536,10 @@
       <c r="K82" s="6">
         <v>1</v>
       </c>
-      <c r="L82" s="5" t="s">
+      <c r="L82" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M82" s="5" t="s">
+      <c r="M82" s="19" t="s">
         <v>458</v>
       </c>
       <c r="N82" s="5"/>
@@ -12586,10 +12593,10 @@
       <c r="K83" s="9">
         <v>1</v>
       </c>
-      <c r="L83" s="8" t="s">
+      <c r="L83" s="20" t="s">
         <v>510</v>
       </c>
-      <c r="M83" s="8" t="s">
+      <c r="M83" s="20" t="s">
         <v>198</v>
       </c>
       <c r="N83" s="8"/>
@@ -12643,10 +12650,10 @@
       <c r="K84" s="6">
         <v>1</v>
       </c>
-      <c r="L84" s="5" t="s">
+      <c r="L84" s="19" t="s">
         <v>510</v>
       </c>
-      <c r="M84" s="5" t="s">
+      <c r="M84" s="19" t="s">
         <v>198</v>
       </c>
       <c r="N84" s="5"/>
@@ -12700,10 +12707,10 @@
       <c r="K85" s="9">
         <v>1</v>
       </c>
-      <c r="L85" s="8" t="s">
+      <c r="L85" s="20" t="s">
         <v>510</v>
       </c>
-      <c r="M85" s="8" t="s">
+      <c r="M85" s="20" t="s">
         <v>198</v>
       </c>
       <c r="N85" s="8"/>
@@ -12757,10 +12764,10 @@
       <c r="K86" s="6">
         <v>1</v>
       </c>
-      <c r="L86" s="5" t="s">
+      <c r="L86" s="19" t="s">
         <v>510</v>
       </c>
-      <c r="M86" s="5" t="s">
+      <c r="M86" s="19" t="s">
         <v>198</v>
       </c>
       <c r="N86" s="5"/>
@@ -12814,10 +12821,10 @@
       <c r="K87" s="9">
         <v>1</v>
       </c>
-      <c r="L87" s="8" t="s">
+      <c r="L87" s="20" t="s">
         <v>510</v>
       </c>
-      <c r="M87" s="8" t="s">
+      <c r="M87" s="20" t="s">
         <v>198</v>
       </c>
       <c r="N87" s="8"/>
@@ -12871,10 +12878,10 @@
       <c r="K88" s="6">
         <v>1</v>
       </c>
-      <c r="L88" s="5" t="s">
+      <c r="L88" s="19" t="s">
         <v>510</v>
       </c>
-      <c r="M88" s="5" t="s">
+      <c r="M88" s="19" t="s">
         <v>198</v>
       </c>
       <c r="N88" s="5"/>
@@ -12928,10 +12935,10 @@
       <c r="K89" s="9">
         <v>1</v>
       </c>
-      <c r="L89" s="8" t="s">
+      <c r="L89" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M89" s="8" t="s">
+      <c r="M89" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N89" s="8"/>
@@ -12985,10 +12992,10 @@
       <c r="K90" s="6">
         <v>1</v>
       </c>
-      <c r="L90" s="5" t="s">
+      <c r="L90" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M90" s="5" t="s">
+      <c r="M90" s="19" t="s">
         <v>458</v>
       </c>
       <c r="N90" s="5"/>
@@ -13042,10 +13049,10 @@
       <c r="K91" s="9">
         <v>1</v>
       </c>
-      <c r="L91" s="8" t="s">
+      <c r="L91" s="20" t="s">
         <v>510</v>
       </c>
-      <c r="M91" s="8" t="s">
+      <c r="M91" s="20" t="s">
         <v>198</v>
       </c>
       <c r="N91" s="8"/>
@@ -13099,10 +13106,10 @@
       <c r="K92" s="6">
         <v>1</v>
       </c>
-      <c r="L92" s="5" t="s">
+      <c r="L92" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M92" s="5" t="s">
+      <c r="M92" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N92" s="5"/>
@@ -13156,10 +13163,10 @@
       <c r="K93" s="9">
         <v>1</v>
       </c>
-      <c r="L93" s="8" t="s">
+      <c r="L93" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M93" s="8" t="s">
+      <c r="M93" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N93" s="8"/>
@@ -13213,10 +13220,10 @@
       <c r="K94" s="6">
         <v>1</v>
       </c>
-      <c r="L94" s="5" t="s">
+      <c r="L94" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="M94" s="5" t="s">
+      <c r="M94" s="19" t="s">
         <v>458</v>
       </c>
       <c r="N94" s="5"/>
@@ -13270,10 +13277,10 @@
       <c r="K95" s="9">
         <v>1</v>
       </c>
-      <c r="L95" s="8" t="s">
+      <c r="L95" s="20" t="s">
         <v>245</v>
       </c>
-      <c r="M95" s="8" t="s">
+      <c r="M95" s="20" t="s">
         <v>458</v>
       </c>
       <c r="N95" s="8"/>
@@ -13327,10 +13334,10 @@
       <c r="K96" s="6">
         <v>1</v>
       </c>
-      <c r="L96" s="5" t="s">
+      <c r="L96" s="19" t="s">
         <v>510</v>
       </c>
-      <c r="M96" s="5" t="s">
+      <c r="M96" s="19" t="s">
         <v>198</v>
       </c>
       <c r="N96" s="5"/>
@@ -13384,10 +13391,10 @@
       <c r="K97" s="9">
         <v>1</v>
       </c>
-      <c r="L97" s="8" t="s">
+      <c r="L97" s="20" t="s">
         <v>510</v>
       </c>
-      <c r="M97" s="8" t="s">
+      <c r="M97" s="20" t="s">
         <v>198</v>
       </c>
       <c r="N97" s="8"/>
@@ -13441,10 +13448,10 @@
       <c r="K98" s="6">
         <v>1</v>
       </c>
-      <c r="L98" s="5" t="s">
+      <c r="L98" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M98" s="5" t="s">
+      <c r="M98" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N98" s="5"/>
@@ -13498,10 +13505,10 @@
       <c r="K99" s="9">
         <v>1</v>
       </c>
-      <c r="L99" s="8" t="s">
+      <c r="L99" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="M99" s="8" t="s">
+      <c r="M99" s="20" t="s">
         <v>199</v>
       </c>
       <c r="N99" s="8"/>
@@ -13555,10 +13562,10 @@
       <c r="K100" s="6">
         <v>1</v>
       </c>
-      <c r="L100" s="5" t="s">
+      <c r="L100" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="M100" s="5" t="s">
+      <c r="M100" s="19" t="s">
         <v>199</v>
       </c>
       <c r="N100" s="5"/>

</xml_diff>